<commit_message>
sweets-ja: not using NLU
</commit_message>
<xml_diff>
--- a/sweets-ja/sweets-ja/scenario.xlsx
+++ b/sweets-ja/sweets-ja/scenario.xlsx
@@ -610,11 +610,7 @@
           <t>はい</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>肯定</t>
-        </is>
-      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>$"ユーザが肯定的な応答をしたかどうかを判断してください。"</t>
@@ -640,11 +636,7 @@
           <t>いいえ</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>否定</t>
-        </is>
-      </c>
+      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>$"ユーザが否定的な応答をしたかどうかを判断してください。"</t>

</xml_diff>